<commit_message>
Reduce store status to 已發送 / 未發送
Replaces the six-step contact status with a binary one driven by the
original spreadsheet's row fill: filled rows start as 已發送, everything
else as 未發送. Drops the 已聯繫 and 已合作 tallies — the header now counts
已發送 / 未發送, and street ratios and the progress bar follow 已發送.

Existing status.json records written under the old scheme are normalized
on load (未聯繫 → 未發送, everything else → 已發送), so filled-in records
survive the change.

Form labels and the Excel builder move from 聯繫 to 發送 wording; the JSON
field names (contactedAt/channel) are left alone to keep the API stable.
Regenerates 澎湖店家確認表單.xlsx: 104 已發送, 222 未發送.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GnsGHJDPPMTcPQobUjM3pp
</commit_message>
<xml_diff>
--- a/澎湖店家確認表單.xlsx
+++ b/澎湖店家確認表單.xlsx
@@ -172,7 +172,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -180,16 +180,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -625,7 +615,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>完成率</t>
+          <t>發送率</t>
         </is>
       </c>
     </row>
@@ -3133,17 +3123,17 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>聯繫狀態</t>
+          <t>發送狀態</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>聯繫日期</t>
+          <t>發送日期</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>聯繫方式</t>
+          <t>發送方式</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -3221,7 +3211,7 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J6" s="14" t="n"/>
@@ -3273,7 +3263,7 @@
       </c>
       <c r="I7" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J7" s="14" t="n"/>
@@ -3321,7 +3311,7 @@
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J8" s="14" t="n"/>
@@ -3369,7 +3359,7 @@
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J9" s="14" t="n"/>
@@ -3417,7 +3407,7 @@
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J10" s="14" t="n"/>
@@ -3465,7 +3455,7 @@
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J11" s="14" t="n"/>
@@ -3513,7 +3503,7 @@
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J12" s="14" t="n"/>
@@ -3565,7 +3555,7 @@
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J13" s="14" t="n"/>
@@ -3617,7 +3607,7 @@
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J14" s="14" t="n"/>
@@ -3725,7 +3715,7 @@
       </c>
       <c r="I16" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J16" s="14" t="n"/>
@@ -3785,7 +3775,7 @@
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J17" s="14" t="n"/>
@@ -4477,7 +4467,7 @@
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J31" s="14" t="n"/>
@@ -4525,7 +4515,7 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J32" s="14" t="n"/>
@@ -4573,7 +4563,7 @@
       </c>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J33" s="14" t="n"/>
@@ -4621,7 +4611,7 @@
       </c>
       <c r="I34" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J34" s="14" t="n"/>
@@ -4981,7 +4971,7 @@
       </c>
       <c r="I41" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J41" s="14" t="n"/>
@@ -5193,7 +5183,7 @@
       </c>
       <c r="I45" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J45" s="14" t="n"/>
@@ -5401,7 +5391,7 @@
       </c>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J49" s="14" t="n"/>
@@ -5457,7 +5447,7 @@
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J50" s="14" t="n"/>
@@ -5641,7 +5631,7 @@
       </c>
       <c r="I54" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J54" s="14" t="n"/>
@@ -5689,7 +5679,7 @@
       </c>
       <c r="I55" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J55" s="14" t="n"/>
@@ -5737,7 +5727,7 @@
       </c>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J56" s="14" t="n"/>
@@ -5785,7 +5775,7 @@
       </c>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J57" s="14" t="n"/>
@@ -5833,7 +5823,7 @@
       </c>
       <c r="I58" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J58" s="14" t="n"/>
@@ -5881,7 +5871,7 @@
       </c>
       <c r="I59" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J59" s="14" t="n"/>
@@ -6685,7 +6675,7 @@
       </c>
       <c r="I75" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J75" s="14" t="n"/>
@@ -6737,7 +6727,7 @@
       </c>
       <c r="I76" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J76" s="14" t="n"/>
@@ -6785,7 +6775,7 @@
       </c>
       <c r="I77" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J77" s="14" t="n"/>
@@ -6837,7 +6827,7 @@
       </c>
       <c r="I78" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J78" s="14" t="n"/>
@@ -6885,7 +6875,7 @@
       </c>
       <c r="I79" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J79" s="14" t="n"/>
@@ -6933,7 +6923,7 @@
       </c>
       <c r="I80" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J80" s="14" t="n"/>
@@ -6981,7 +6971,7 @@
       </c>
       <c r="I81" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J81" s="14" t="n"/>
@@ -7029,7 +7019,7 @@
       </c>
       <c r="I82" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J82" s="14" t="n"/>
@@ -7081,7 +7071,7 @@
       </c>
       <c r="I83" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J83" s="14" t="n"/>
@@ -7133,7 +7123,7 @@
       </c>
       <c r="I84" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J84" s="14" t="n"/>
@@ -7193,7 +7183,7 @@
       </c>
       <c r="I85" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J85" s="14" t="n"/>
@@ -7249,7 +7239,7 @@
       </c>
       <c r="I86" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J86" s="14" t="n"/>
@@ -7305,7 +7295,7 @@
       </c>
       <c r="I87" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J87" s="14" t="n"/>
@@ -7385,7 +7375,7 @@
       </c>
       <c r="I89" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J89" s="14" t="n"/>
@@ -7441,7 +7431,7 @@
       </c>
       <c r="I90" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J90" s="14" t="n"/>
@@ -7493,7 +7483,7 @@
       </c>
       <c r="I91" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J91" s="14" t="n"/>
@@ -7541,7 +7531,7 @@
       </c>
       <c r="I92" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J92" s="14" t="n"/>
@@ -7589,7 +7579,7 @@
       </c>
       <c r="I93" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J93" s="14" t="n"/>
@@ -7637,7 +7627,7 @@
       </c>
       <c r="I94" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J94" s="14" t="n"/>
@@ -7685,7 +7675,7 @@
       </c>
       <c r="I95" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J95" s="14" t="n"/>
@@ -7733,7 +7723,7 @@
       </c>
       <c r="I96" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J96" s="14" t="n"/>
@@ -7781,7 +7771,7 @@
       </c>
       <c r="I97" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J97" s="14" t="n"/>
@@ -7833,7 +7823,7 @@
       </c>
       <c r="I98" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J98" s="14" t="n"/>
@@ -7889,7 +7879,7 @@
       </c>
       <c r="I99" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J99" s="14" t="n"/>
@@ -7945,7 +7935,7 @@
       </c>
       <c r="I100" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J100" s="14" t="n"/>
@@ -8073,7 +8063,7 @@
       </c>
       <c r="I103" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J103" s="14" t="n"/>
@@ -8169,7 +8159,7 @@
       </c>
       <c r="I105" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J105" s="14" t="n"/>
@@ -8217,7 +8207,7 @@
       </c>
       <c r="I106" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J106" s="14" t="n"/>
@@ -8265,7 +8255,7 @@
       </c>
       <c r="I107" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J107" s="14" t="n"/>
@@ -8313,7 +8303,7 @@
       </c>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J108" s="14" t="n"/>
@@ -8409,7 +8399,7 @@
       </c>
       <c r="I110" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J110" s="14" t="n"/>
@@ -8457,7 +8447,7 @@
       </c>
       <c r="I111" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J111" s="14" t="n"/>
@@ -8505,7 +8495,7 @@
       </c>
       <c r="I112" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J112" s="14" t="n"/>
@@ -8553,7 +8543,7 @@
       </c>
       <c r="I113" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J113" s="14" t="n"/>
@@ -8605,7 +8595,7 @@
       </c>
       <c r="I114" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J114" s="14" t="n"/>
@@ -8681,7 +8671,7 @@
       </c>
       <c r="I116" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J116" s="14" t="n"/>
@@ -8729,7 +8719,7 @@
       </c>
       <c r="I117" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J117" s="14" t="n"/>
@@ -8777,7 +8767,7 @@
       </c>
       <c r="I118" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J118" s="14" t="n"/>
@@ -8825,7 +8815,7 @@
       </c>
       <c r="I119" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J119" s="14" t="n"/>
@@ -8873,7 +8863,7 @@
       </c>
       <c r="I120" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J120" s="14" t="n"/>
@@ -9129,7 +9119,7 @@
       </c>
       <c r="I125" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J125" s="14" t="n"/>
@@ -9314,7 +9304,7 @@
       </c>
       <c r="I129" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J129" s="14" t="n"/>
@@ -9366,7 +9356,7 @@
       </c>
       <c r="I130" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J130" s="14" t="n"/>
@@ -9414,7 +9404,7 @@
       </c>
       <c r="I131" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J131" s="14" t="n"/>
@@ -9462,7 +9452,7 @@
       </c>
       <c r="I132" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J132" s="14" t="n"/>
@@ -9510,7 +9500,7 @@
       </c>
       <c r="I133" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J133" s="14" t="n"/>
@@ -9558,7 +9548,7 @@
       </c>
       <c r="I134" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J134" s="14" t="n"/>
@@ -9674,7 +9664,7 @@
       </c>
       <c r="I136" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J136" s="14" t="n"/>
@@ -9734,7 +9724,7 @@
       </c>
       <c r="I137" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J137" s="14" t="n"/>
@@ -9846,7 +9836,7 @@
       </c>
       <c r="I139" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J139" s="14" t="n"/>
@@ -9918,7 +9908,7 @@
       </c>
       <c r="I141" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J141" s="14" t="n"/>
@@ -9970,7 +9960,7 @@
       </c>
       <c r="I142" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J142" s="14" t="n"/>
@@ -10018,7 +10008,7 @@
       </c>
       <c r="I143" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J143" s="14" t="n"/>
@@ -10066,7 +10056,7 @@
       </c>
       <c r="I144" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J144" s="14" t="n"/>
@@ -10114,7 +10104,7 @@
       </c>
       <c r="I145" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J145" s="14" t="n"/>
@@ -10162,7 +10152,7 @@
       </c>
       <c r="I146" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J146" s="14" t="n"/>
@@ -10210,7 +10200,7 @@
       </c>
       <c r="I147" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J147" s="14" t="n"/>
@@ -10258,7 +10248,7 @@
       </c>
       <c r="I148" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J148" s="14" t="n"/>
@@ -10310,7 +10300,7 @@
       </c>
       <c r="I149" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J149" s="14" t="n"/>
@@ -10362,7 +10352,7 @@
       </c>
       <c r="I150" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J150" s="14" t="n"/>
@@ -10430,7 +10420,7 @@
       </c>
       <c r="I152" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J152" s="14" t="n"/>
@@ -10478,7 +10468,7 @@
       </c>
       <c r="I153" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J153" s="14" t="n"/>
@@ -10526,7 +10516,7 @@
       </c>
       <c r="I154" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J154" s="14" t="n"/>
@@ -10578,7 +10568,7 @@
       </c>
       <c r="I155" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J155" s="14" t="n"/>
@@ -10634,7 +10624,7 @@
       </c>
       <c r="I156" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J156" s="14" t="n"/>
@@ -10966,7 +10956,7 @@
       </c>
       <c r="I163" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J163" s="14" t="n"/>
@@ -11022,7 +11012,7 @@
       </c>
       <c r="I164" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J164" s="14" t="n"/>
@@ -11070,7 +11060,7 @@
       </c>
       <c r="I165" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J165" s="14" t="n"/>
@@ -11118,7 +11108,7 @@
       </c>
       <c r="I166" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J166" s="14" t="n"/>
@@ -11166,7 +11156,7 @@
       </c>
       <c r="I167" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J167" s="14" t="n"/>
@@ -11214,7 +11204,7 @@
       </c>
       <c r="I168" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J168" s="14" t="n"/>
@@ -11266,7 +11256,7 @@
       </c>
       <c r="I169" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J169" s="14" t="n"/>
@@ -11314,7 +11304,7 @@
       </c>
       <c r="I170" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J170" s="14" t="n"/>
@@ -11386,7 +11376,7 @@
       </c>
       <c r="I172" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J172" s="14" t="n"/>
@@ -11434,7 +11424,7 @@
       </c>
       <c r="I173" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J173" s="14" t="n"/>
@@ -11482,7 +11472,7 @@
       </c>
       <c r="I174" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J174" s="14" t="n"/>
@@ -11762,7 +11752,7 @@
       </c>
       <c r="I180" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J180" s="14" t="n"/>
@@ -11810,7 +11800,7 @@
       </c>
       <c r="I181" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J181" s="14" t="n"/>
@@ -11858,7 +11848,7 @@
       </c>
       <c r="I182" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J182" s="14" t="n"/>
@@ -11906,7 +11896,7 @@
       </c>
       <c r="I183" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J183" s="14" t="n"/>
@@ -12062,7 +12052,7 @@
       </c>
       <c r="I186" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J186" s="14" t="n"/>
@@ -12138,7 +12128,7 @@
       </c>
       <c r="I188" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J188" s="14" t="n"/>
@@ -12238,7 +12228,7 @@
       </c>
       <c r="I190" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J190" s="14" t="n"/>
@@ -12342,7 +12332,7 @@
       </c>
       <c r="I192" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J192" s="14" t="n"/>
@@ -12398,7 +12388,7 @@
       </c>
       <c r="I193" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J193" s="14" t="n"/>
@@ -12674,7 +12664,7 @@
       </c>
       <c r="I199" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J199" s="14" t="n"/>
@@ -12746,7 +12736,7 @@
       </c>
       <c r="I201" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J201" s="14" t="n"/>
@@ -12794,7 +12784,7 @@
       </c>
       <c r="I202" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J202" s="14" t="n"/>
@@ -12842,7 +12832,7 @@
       </c>
       <c r="I203" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J203" s="14" t="n"/>
@@ -12890,7 +12880,7 @@
       </c>
       <c r="I204" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J204" s="14" t="n"/>
@@ -12942,7 +12932,7 @@
       </c>
       <c r="I205" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J205" s="14" t="n"/>
@@ -13010,7 +13000,7 @@
       </c>
       <c r="I207" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J207" s="14" t="n"/>
@@ -13062,7 +13052,7 @@
       </c>
       <c r="I208" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J208" s="14" t="n"/>
@@ -13114,7 +13104,7 @@
       </c>
       <c r="I209" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J209" s="14" t="n"/>
@@ -13166,7 +13156,7 @@
       </c>
       <c r="I210" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J210" s="14" t="n"/>
@@ -13222,7 +13212,7 @@
       </c>
       <c r="I211" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J211" s="14" t="n"/>
@@ -13354,7 +13344,7 @@
       </c>
       <c r="I214" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J214" s="14" t="n"/>
@@ -13406,7 +13396,7 @@
       </c>
       <c r="I215" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J215" s="14" t="n"/>
@@ -13462,7 +13452,7 @@
       </c>
       <c r="I216" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J216" s="14" t="n"/>
@@ -13766,7 +13756,7 @@
       </c>
       <c r="I223" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J223" s="14" t="n"/>
@@ -13866,7 +13856,7 @@
       </c>
       <c r="I225" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J225" s="14" t="n"/>
@@ -13994,7 +13984,7 @@
       </c>
       <c r="I228" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J228" s="14" t="n"/>
@@ -14042,7 +14032,7 @@
       </c>
       <c r="I229" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J229" s="14" t="n"/>
@@ -14222,7 +14212,7 @@
       </c>
       <c r="I233" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J233" s="14" t="n"/>
@@ -14270,7 +14260,7 @@
       </c>
       <c r="I234" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J234" s="14" t="n"/>
@@ -14318,7 +14308,7 @@
       </c>
       <c r="I235" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J235" s="14" t="n"/>
@@ -14386,7 +14376,7 @@
       </c>
       <c r="I237" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J237" s="14" t="n"/>
@@ -14434,7 +14424,7 @@
       </c>
       <c r="I238" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J238" s="14" t="n"/>
@@ -14482,7 +14472,7 @@
       </c>
       <c r="I239" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J239" s="14" t="n"/>
@@ -14554,7 +14544,7 @@
       </c>
       <c r="I241" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J241" s="14" t="n"/>
@@ -14602,7 +14592,7 @@
       </c>
       <c r="I242" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J242" s="14" t="n"/>
@@ -14650,7 +14640,7 @@
       </c>
       <c r="I243" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J243" s="14" t="n"/>
@@ -14718,7 +14708,7 @@
       </c>
       <c r="I245" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J245" s="14" t="n"/>
@@ -14766,7 +14756,7 @@
       </c>
       <c r="I246" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J246" s="14" t="n"/>
@@ -14822,7 +14812,7 @@
       </c>
       <c r="I247" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J247" s="14" t="n"/>
@@ -14894,7 +14884,7 @@
       </c>
       <c r="I249" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J249" s="14" t="n"/>
@@ -14942,7 +14932,7 @@
       </c>
       <c r="I250" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J250" s="14" t="n"/>
@@ -14998,7 +14988,7 @@
       </c>
       <c r="I251" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J251" s="14" t="n"/>
@@ -15114,7 +15104,7 @@
       </c>
       <c r="I254" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J254" s="14" t="n"/>
@@ -15162,7 +15152,7 @@
       </c>
       <c r="I255" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J255" s="14" t="n"/>
@@ -15230,7 +15220,7 @@
       </c>
       <c r="I257" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J257" s="14" t="n"/>
@@ -15278,7 +15268,7 @@
       </c>
       <c r="I258" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J258" s="14" t="n"/>
@@ -15398,7 +15388,7 @@
       </c>
       <c r="I261" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J261" s="14" t="n"/>
@@ -15578,7 +15568,7 @@
       </c>
       <c r="I265" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J265" s="14" t="n"/>
@@ -15626,7 +15616,7 @@
       </c>
       <c r="I266" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J266" s="14" t="n"/>
@@ -15686,7 +15676,7 @@
       </c>
       <c r="I267" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J267" s="14" t="n"/>
@@ -15754,7 +15744,7 @@
       </c>
       <c r="I269" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J269" s="14" t="n"/>
@@ -15802,7 +15792,7 @@
       </c>
       <c r="I270" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J270" s="14" t="n"/>
@@ -15850,7 +15840,7 @@
       </c>
       <c r="I271" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J271" s="14" t="n"/>
@@ -15918,7 +15908,7 @@
       </c>
       <c r="I273" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J273" s="14" t="n"/>
@@ -15970,7 +15960,7 @@
       </c>
       <c r="I274" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J274" s="14" t="n"/>
@@ -16018,7 +16008,7 @@
       </c>
       <c r="I275" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J275" s="14" t="n"/>
@@ -16146,7 +16136,7 @@
       </c>
       <c r="I278" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J278" s="14" t="n"/>
@@ -16198,7 +16188,7 @@
       </c>
       <c r="I279" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J279" s="14" t="n"/>
@@ -16330,7 +16320,7 @@
       </c>
       <c r="I282" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J282" s="14" t="n"/>
@@ -16398,7 +16388,7 @@
       </c>
       <c r="I284" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J284" s="14" t="n"/>
@@ -16446,7 +16436,7 @@
       </c>
       <c r="I285" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J285" s="14" t="n"/>
@@ -16514,7 +16504,7 @@
       </c>
       <c r="I287" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J287" s="14" t="n"/>
@@ -16638,7 +16628,7 @@
       </c>
       <c r="I290" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J290" s="14" t="n"/>
@@ -16686,7 +16676,7 @@
       </c>
       <c r="I291" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J291" s="14" t="n"/>
@@ -16754,7 +16744,7 @@
       </c>
       <c r="I293" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J293" s="14" t="n"/>
@@ -16802,7 +16792,7 @@
       </c>
       <c r="I294" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J294" s="14" t="n"/>
@@ -16870,7 +16860,7 @@
       </c>
       <c r="I296" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J296" s="14" t="n"/>
@@ -16918,7 +16908,7 @@
       </c>
       <c r="I297" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J297" s="14" t="n"/>
@@ -16986,7 +16976,7 @@
       </c>
       <c r="I299" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J299" s="14" t="n"/>
@@ -17034,7 +17024,7 @@
       </c>
       <c r="I300" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J300" s="14" t="n"/>
@@ -17102,7 +17092,7 @@
       </c>
       <c r="I302" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J302" s="14" t="n"/>
@@ -17222,7 +17212,7 @@
       </c>
       <c r="I305" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J305" s="14" t="n"/>
@@ -17270,7 +17260,7 @@
       </c>
       <c r="I306" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J306" s="14" t="n"/>
@@ -17338,7 +17328,7 @@
       </c>
       <c r="I308" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J308" s="14" t="n"/>
@@ -17386,7 +17376,7 @@
       </c>
       <c r="I309" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J309" s="14" t="n"/>
@@ -17454,7 +17444,7 @@
       </c>
       <c r="I311" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J311" s="14" t="n"/>
@@ -17578,7 +17568,7 @@
       </c>
       <c r="I314" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J314" s="14" t="n"/>
@@ -17626,7 +17616,7 @@
       </c>
       <c r="I315" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J315" s="14" t="n"/>
@@ -17818,7 +17808,7 @@
       </c>
       <c r="I320" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J320" s="14" t="n"/>
@@ -17894,7 +17884,7 @@
       </c>
       <c r="I322" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J322" s="14" t="n"/>
@@ -17966,7 +17956,7 @@
       </c>
       <c r="I324" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J324" s="14" t="n"/>
@@ -18034,7 +18024,7 @@
       </c>
       <c r="I326" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J326" s="14" t="n"/>
@@ -18106,7 +18096,7 @@
       </c>
       <c r="I328" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J328" s="14" t="n"/>
@@ -18174,7 +18164,7 @@
       </c>
       <c r="I330" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J330" s="14" t="n"/>
@@ -18246,7 +18236,7 @@
       </c>
       <c r="I332" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J332" s="14" t="n"/>
@@ -18314,7 +18304,7 @@
       </c>
       <c r="I334" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J334" s="14" t="n"/>
@@ -18382,7 +18372,7 @@
       </c>
       <c r="I336" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J336" s="14" t="n"/>
@@ -18450,7 +18440,7 @@
       </c>
       <c r="I338" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J338" s="14" t="n"/>
@@ -18518,7 +18508,7 @@
       </c>
       <c r="I340" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J340" s="14" t="n"/>
@@ -18586,7 +18576,7 @@
       </c>
       <c r="I342" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J342" s="14" t="n"/>
@@ -18722,7 +18712,7 @@
       </c>
       <c r="I346" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J346" s="14" t="n"/>
@@ -18794,7 +18784,7 @@
       </c>
       <c r="I348" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J348" s="14" t="n"/>
@@ -18866,7 +18856,7 @@
       </c>
       <c r="I350" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J350" s="14" t="n"/>
@@ -18943,7 +18933,7 @@
       </c>
       <c r="I352" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J352" s="14" t="n"/>
@@ -19011,7 +19001,7 @@
       </c>
       <c r="I354" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J354" s="14" t="n"/>
@@ -19079,7 +19069,7 @@
       </c>
       <c r="I356" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J356" s="14" t="n"/>
@@ -19147,7 +19137,7 @@
       </c>
       <c r="I358" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J358" s="14" t="n"/>
@@ -19219,7 +19209,7 @@
       </c>
       <c r="I360" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J360" s="14" t="n"/>
@@ -19287,7 +19277,7 @@
       </c>
       <c r="I362" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J362" s="14" t="n"/>
@@ -19355,7 +19345,7 @@
       </c>
       <c r="I364" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J364" s="14" t="n"/>
@@ -19423,7 +19413,7 @@
       </c>
       <c r="I366" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J366" s="14" t="n"/>
@@ -19491,7 +19481,7 @@
       </c>
       <c r="I368" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J368" s="14" t="n"/>
@@ -19559,7 +19549,7 @@
       </c>
       <c r="I370" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J370" s="14" t="n"/>
@@ -19859,7 +19849,7 @@
       </c>
       <c r="I377" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J377" s="14" t="n"/>
@@ -20267,7 +20257,7 @@
       </c>
       <c r="I386" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J386" s="14" t="n"/>
@@ -20339,7 +20329,7 @@
       </c>
       <c r="I388" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J388" s="14" t="n"/>
@@ -20459,7 +20449,7 @@
       </c>
       <c r="I391" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J391" s="14" t="n"/>
@@ -20527,7 +20517,7 @@
       </c>
       <c r="I393" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J393" s="14" t="n"/>
@@ -20603,7 +20593,7 @@
       </c>
       <c r="I395" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J395" s="14" t="n"/>
@@ -20675,7 +20665,7 @@
       </c>
       <c r="I397" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J397" s="14" t="n"/>
@@ -20743,7 +20733,7 @@
       </c>
       <c r="I399" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J399" s="14" t="n"/>
@@ -20967,7 +20957,7 @@
       </c>
       <c r="I405" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J405" s="14" t="n"/>
@@ -21019,7 +21009,7 @@
       </c>
       <c r="I406" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J406" s="14" t="n"/>
@@ -21071,7 +21061,7 @@
       </c>
       <c r="I407" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J407" s="14" t="n"/>
@@ -21147,7 +21137,7 @@
       </c>
       <c r="I409" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J409" s="14" t="n"/>
@@ -21219,7 +21209,7 @@
       </c>
       <c r="I411" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J411" s="14" t="n"/>
@@ -21287,7 +21277,7 @@
       </c>
       <c r="I413" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J413" s="14" t="n"/>
@@ -21427,7 +21417,7 @@
       </c>
       <c r="I417" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J417" s="14" t="n"/>
@@ -21499,7 +21489,7 @@
       </c>
       <c r="I419" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J419" s="14" t="n"/>
@@ -21575,7 +21565,7 @@
       </c>
       <c r="I421" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J421" s="14" t="n"/>
@@ -21627,7 +21617,7 @@
       </c>
       <c r="I422" s="13" t="inlineStr">
         <is>
-          <t>未聯繫</t>
+          <t>未發送</t>
         </is>
       </c>
       <c r="J422" s="14" t="n"/>
@@ -21734,18 +21724,15 @@
   </mergeCells>
   <conditionalFormatting sqref="I6:I29 I31:I52 I54:I73 I75:I87 I89:I101 I103:I114 I116:I127 I129:I139 I141:I150 I152:I161 I163:I170 I172:I178 I180:I186 I188:I193 I195:I199 I201:I205 I207:I211 I213:I216 I218:I221 I223:I226 I228:I231 I233:I235 I237:I239 I241:I243 I245:I247 I249:I251 I253:I255 I257:I259 I261:I263 I265:I267 I269:I271 I273:I275 I277:I279 I281:I282 I284:I285 I287:I288 I290:I291 I293:I294 I296:I297 I299:I300 I302:I303 I305:I306 I308:I309 I311:I312 I314:I315 I317:I318 I320 I322 I324 I326 I328 I330 I332 I334 I336 I338 I340 I342 I344 I346 I348 I350 I352 I354 I356 I358 I360 I362 I364 I366 I368 I370:I371 I373 I375:I378 I380:I383 I385:I386 I388:I389 I391 I393 I395 I397 I399 I401 I403 I405:I407 I409 I411 I413 I415 I417 I419 I421:I422">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"已合作"</formula>
+      <formula>"已發送"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"婉拒"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
-      <formula>"聯繫不上"</formula>
+      <formula>"未發送"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="I6:I29 I31:I52 I54:I73 I75:I87 I89:I101 I103:I114 I116:I127 I129:I139 I141:I150 I152:I161 I163:I170 I172:I178 I180:I186 I188:I193 I195:I199 I201:I205 I207:I211 I213:I216 I218:I221 I223:I226 I228:I231 I233:I235 I237:I239 I241:I243 I245:I247 I249:I251 I253:I255 I257:I259 I261:I263 I265:I267 I269:I271 I273:I275 I277:I279 I281:I282 I284:I285 I287:I288 I290:I291 I293:I294 I296:I297 I299:I300 I302:I303 I305:I306 I308:I309 I311:I312 I314:I315 I317:I318 I320 I322 I324 I326 I328 I330 I332 I334 I336 I338 I340 I342 I344 I346 I348 I350 I352 I354 I356 I358 I360 I362 I364 I366 I368 I370:I371 I373 I375:I378 I380:I383 I385:I386 I388:I389 I391 I393 I395 I397 I399 I401 I403 I405:I407 I409 I411 I413 I415 I417 I419 I421:I422" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"未聯繫,已發送,已回覆,已合作,婉拒,聯繫不上"</formula1>
+      <formula1>"未發送,已發送"</formula1>
     </dataValidation>
     <dataValidation sqref="K6:K29 K31:K52 K54:K73 K75:K87 K89:K101 K103:K114 K116:K127 K129:K139 K141:K150 K152:K161 K163:K170 K172:K178 K180:K186 K188:K193 K195:K199 K201:K205 K207:K211 K213:K216 K218:K221 K223:K226 K228:K231 K233:K235 K237:K239 K241:K243 K245:K247 K249:K251 K253:K255 K257:K259 K261:K263 K265:K267 K269:K271 K273:K275 K277:K279 K281:K282 K284:K285 K287:K288 K290:K291 K293:K294 K296:K297 K299:K300 K302:K303 K305:K306 K308:K309 K311:K312 K314:K315 K317:K318 K320 K322 K324 K326 K328 K330 K332 K334 K336 K338 K340 K342 K344 K346 K348 K350 K352 K354 K356 K358 K360 K362 K364 K366 K368 K370:K371 K373 K375:K378 K380:K383 K385:K386 K388:K389 K391 K393 K395 K397 K399 K401 K403 K405:K407 K409 K411 K413 K415 K417 K419 K421:K422" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"現場拜訪,電話,LINE,Email,FB/IG 私訊"</formula1>
@@ -21809,7 +21796,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>聯繫狀態</t>
+          <t>發送狀態</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -23038,7 +23025,7 @@
   <autoFilter ref="A4:F80"/>
   <dataValidations count="1">
     <dataValidation sqref="E5:E80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"未聯繫,已發送,已回覆,已合作,婉拒,聯繫不上"</formula1>
+      <formula1>"未發送,已發送"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 已張貼 as a third status after 已發送
Status becomes 未發送 → 已發送 → 已張貼 on both the main list and the
新增家數 page, and in the confirmation spreadsheet's dropdown.

Progress bars and per-street ratios now count 已處理 — anything that is not
未發送 — so a store moving from 已發送 to 已張貼 no longer drops out of the
count. The header breaks the three states out into their own tiles, which
now wrap on narrow screens instead of sitting in a fixed four-column grid.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GnsGHJDPPMTcPQobUjM3pp
</commit_message>
<xml_diff>
--- a/澎湖店家確認表單.xlsx
+++ b/澎湖店家確認表單.xlsx
@@ -172,7 +172,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -180,6 +180,16 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -21724,15 +21734,18 @@
   </mergeCells>
   <conditionalFormatting sqref="I6:I29 I31:I52 I54:I73 I75:I87 I89:I101 I103:I114 I116:I127 I129:I139 I141:I150 I152:I161 I163:I170 I172:I178 I180:I186 I188:I193 I195:I199 I201:I205 I207:I211 I213:I216 I218:I221 I223:I226 I228:I231 I233:I235 I237:I239 I241:I243 I245:I247 I249:I251 I253:I255 I257:I259 I261:I263 I265:I267 I269:I271 I273:I275 I277:I279 I281:I282 I284:I285 I287:I288 I290:I291 I293:I294 I296:I297 I299:I300 I302:I303 I305:I306 I308:I309 I311:I312 I314:I315 I317:I318 I320 I322 I324 I326 I328 I330 I332 I334 I336 I338 I340 I342 I344 I346 I348 I350 I352 I354 I356 I358 I360 I362 I364 I366 I368 I370:I371 I373 I375:I378 I380:I383 I385:I386 I388:I389 I391 I393 I395 I397 I399 I401 I403 I405:I407 I409 I411 I413 I415 I417 I419 I421:I422">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"已張貼"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
       <formula>"已發送"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"未發送"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="I6:I29 I31:I52 I54:I73 I75:I87 I89:I101 I103:I114 I116:I127 I129:I139 I141:I150 I152:I161 I163:I170 I172:I178 I180:I186 I188:I193 I195:I199 I201:I205 I207:I211 I213:I216 I218:I221 I223:I226 I228:I231 I233:I235 I237:I239 I241:I243 I245:I247 I249:I251 I253:I255 I257:I259 I261:I263 I265:I267 I269:I271 I273:I275 I277:I279 I281:I282 I284:I285 I287:I288 I290:I291 I293:I294 I296:I297 I299:I300 I302:I303 I305:I306 I308:I309 I311:I312 I314:I315 I317:I318 I320 I322 I324 I326 I328 I330 I332 I334 I336 I338 I340 I342 I344 I346 I348 I350 I352 I354 I356 I358 I360 I362 I364 I366 I368 I370:I371 I373 I375:I378 I380:I383 I385:I386 I388:I389 I391 I393 I395 I397 I399 I401 I403 I405:I407 I409 I411 I413 I415 I417 I419 I421:I422" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"未發送,已發送"</formula1>
+      <formula1>"未發送,已發送,已張貼"</formula1>
     </dataValidation>
     <dataValidation sqref="K6:K29 K31:K52 K54:K73 K75:K87 K89:K101 K103:K114 K116:K127 K129:K139 K141:K150 K152:K161 K163:K170 K172:K178 K180:K186 K188:K193 K195:K199 K201:K205 K207:K211 K213:K216 K218:K221 K223:K226 K228:K231 K233:K235 K237:K239 K241:K243 K245:K247 K249:K251 K253:K255 K257:K259 K261:K263 K265:K267 K269:K271 K273:K275 K277:K279 K281:K282 K284:K285 K287:K288 K290:K291 K293:K294 K296:K297 K299:K300 K302:K303 K305:K306 K308:K309 K311:K312 K314:K315 K317:K318 K320 K322 K324 K326 K328 K330 K332 K334 K336 K338 K340 K342 K344 K346 K348 K350 K352 K354 K356 K358 K360 K362 K364 K366 K368 K370:K371 K373 K375:K378 K380:K383 K385:K386 K388:K389 K391 K393 K395 K397 K399 K401 K403 K405:K407 K409 K411 K413 K415 K417 K419 K421:K422" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"現場拜訪,電話,LINE,Email,FB/IG 私訊"</formula1>
@@ -23025,7 +23038,7 @@
   <autoFilter ref="A4:F80"/>
   <dataValidations count="1">
     <dataValidation sqref="E5:E80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"未發送,已發送"</formula1>
+      <formula1>"未發送,已發送,已張貼"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>